<commit_message>
log cantidad de controles
</commit_message>
<xml_diff>
--- a/Cambiar Lotes/ListaMuestras.xlsx
+++ b/Cambiar Lotes/ListaMuestras.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$B$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$B$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,86 +457,46 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1587258</v>
+        <v>2101000</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>LISTA REPROCESADA</t>
+          <t>PARA DESCARGAR</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1587257</v>
+        <v>2112688</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LISTA REPROCESADA</t>
+          <t>PARA DESCARGAR</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1587255</v>
+        <v>2112049</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LISTA REPROCESADA</t>
+          <t>PARA DESCARGAR</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1587249</v>
+        <v>2148293</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LISTA REPROCESADA</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>1587242</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>LISTA REPROCESADA</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>1587236</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>LISTA REPROCESADA</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>1587232</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>LISTA REPROCESADA</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>1587231</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>LISTA REPROCESADA</t>
+          <t>PARA DESCARGAR</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B9"/>
+  <autoFilter ref="A1:B5"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Pausa en Creación Envase
</commit_message>
<xml_diff>
--- a/Cambiar Lotes/ListaMuestras.xlsx
+++ b/Cambiar Lotes/ListaMuestras.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$B$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$B$264</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B264"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,296 +457,2636 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2403938</v>
+        <v>1769063</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2403939</v>
+        <v>1973986</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2404240</v>
+        <v>2034418</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2404241</v>
+        <v>2034419</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2404242</v>
+        <v>2034420</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2404243</v>
+        <v>2034421</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2404244</v>
+        <v>2034422</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2404359</v>
+        <v>2034423</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2404361</v>
+        <v>2068792</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2404362</v>
+        <v>2084531</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>2404363</v>
+        <v>2175776</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2404364</v>
+        <v>2175777</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2404365</v>
+        <v>2175778</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2404366</v>
+        <v>2175779</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2404367</v>
+        <v>2175780</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>2404368</v>
+        <v>2175781</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2404369</v>
+        <v>2320099</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2404370</v>
+        <v>2320100</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>2404371</v>
+        <v>2320101</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>2404372</v>
+        <v>2320102</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2404373</v>
+        <v>2320103</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>2404374</v>
+        <v>2320104</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>2404375</v>
+        <v>2320105</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2404376</v>
+        <v>2320106</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>2404377</v>
+        <v>2320107</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>2404378</v>
+        <v>2320108</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>2404379</v>
+        <v>2320109</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>2404380</v>
+        <v>2320110</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>2404381</v>
+        <v>2320136</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>2404382</v>
+        <v>2320137</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>2404383</v>
+        <v>2320138</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>2404424</v>
+        <v>2320139</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>2404425</v>
+        <v>2320140</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ANALISIS YA EXISTE</t>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>2320141</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>2320280</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>2320281</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>2320282</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>2320283</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>2320284</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>2320285</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>2320286</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>2320287</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>2320288</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>2320289</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>2320290</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>2320291</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>2321660</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>2321661</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>2321662</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>2321663</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>2321664</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>2321665</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>2336151</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>2349677</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>2360073</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>2362863</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>2367064</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>2367065</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>2367066</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>2367067</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>2367068</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>2376322</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>2376323</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>2376330</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>2380371</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>2380372</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>2380373</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>2380374</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>2380376</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>2380377</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>2380437</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>2380439</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>2380440</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>2380441</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>2380442</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>2380444</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>2380547</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>2380551</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>2380553</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>2380555</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>2380557</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>2380559</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>2380563</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>2380564</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>2380565</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>2380567</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>2380568</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>2380569</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>2380580</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>2380581</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>2380582</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>2380584</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>2380585</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>2380587</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>2380591</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>2380592</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>2380593</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>2380594</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>2380596</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>2380597</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>2380631</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>2380632</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>2380633</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>2380634</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>2380635</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>2380636</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>2380637</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>2380638</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>2380639</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>2380640</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>2380641</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>2380642</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>2380644</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>2380645</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>2380646</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>2380648</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>2380649</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>2380650</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>2380654</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>2380655</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>2380656</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>2380657</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>2380658</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>2380660</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>2380661</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>2380663</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>2380664</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>2380665</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>2380666</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>2380667</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>2380670</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>2380671</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>2380672</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>2380673</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>2380674</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>2380675</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>2380695</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>2380698</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>2380701</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>2380703</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>2380706</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>2380708</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>2380720</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>2380721</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>2380722</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>2380723</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>2380724</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>2380725</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>2380726</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>2380727</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>2380728</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>2380729</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>2380730</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>2380731</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>2380758</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>2380759</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>2380760</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>2380761</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>2380763</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>2380764</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>2380819</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>2380820</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>2380821</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>2380822</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>2380823</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>2380824</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>2380829</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>2380830</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>2380831</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>2380832</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>2380833</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>2380834</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>2380873</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>2380874</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>2380875</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>2380876</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>2380877</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>2380878</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>2425134</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>2443610</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>2444547</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>2450873</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>2450874</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>2450875</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>2450876</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>2451673</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>2451674</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>2453552</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>2453712</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>2453713</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>2453714</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>2453715</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>2453716</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>2453717</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>2453718</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>2453720</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>2453768</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>2453769</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>2453770</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>2453771</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>2453780</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>2453781</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>2453782</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>2453783</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>2453784</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>2453785</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>2453786</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>2453787</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>2453788</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>2453789</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>2453790</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>2453791</v>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>2453792</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>2453793</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>2453794</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="n">
+        <v>2453795</v>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="n">
+        <v>2453796</v>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="n">
+        <v>2453797</v>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="n">
+        <v>2453798</v>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>2453800</v>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
+        <v>2453802</v>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>2453803</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="n">
+        <v>2453804</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>2453805</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>2453806</v>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="n">
+        <v>2453807</v>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>2453808</v>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="n">
+        <v>2453809</v>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>2454209</v>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="n">
+        <v>2455282</v>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>2458794</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>2464095</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>2464230</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>2464234</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>2309589</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>2309570</v>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>2320509</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>1913239</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>2467863</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>2467864</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>2467865</v>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>2467866</v>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="n">
+        <v>2467867</v>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="n">
+        <v>2467868</v>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="n">
+        <v>2467941</v>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="n">
+        <v>2467944</v>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>2467948</v>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="n">
+        <v>2467950</v>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="n">
+        <v>2467952</v>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="n">
+        <v>2467954</v>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="n">
+        <v>2468117</v>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="n">
+        <v>2468118</v>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="n">
+        <v>2468119</v>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="n">
+        <v>2468120</v>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="n">
+        <v>2468121</v>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="n">
+        <v>2468122</v>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="n">
+        <v>2468649</v>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="n">
+        <v>2468684</v>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="n">
+        <v>2468685</v>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>2468686</v>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>2468687</v>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>2468688</v>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>2468689</v>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>EDITADO</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B34"/>
+  <autoFilter ref="A1:B264"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>